<commit_message>
feat(partners): Tasklet fastlane — seal RAKTA/Bahrain MOTC, India consumer brief markets
Merge PR #62/#63 handoffs and run grok/execute_tasklet_fastlane:
- Seal 6 RAKTA + 7 Bahrain MOTC spine corridors to live route_ids
- Mark Kolkata/Chennai brief markets held-null on Ola/Rapido/Uber (no Atlas IDs yet)
- Partner page lane PASS for rakta; Rapido/Ola PASS with 6-market footprint
- Add run_tasklet_fastlane.sh orchestrator
</commit_message>
<xml_diff>
--- a/finance/_partner-tracker.xlsx
+++ b/finance/_partner-tracker.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P53"/>
+  <dimension ref="A1:P55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -633,24 +633,24 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Bahrain MOTC</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>hong-kong</t>
+          <t>bahrain-motc</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>destination_region</t>
+          <t>Authority / national transport</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>East Asia</t>
+          <t>Bahrain / Gulf</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>hong-kong, macau-china</t>
+          <t>manama-bahrain, eastern-province-ksa, doha-qatar, dubai-uae, abu-dhabi-uae</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -690,14 +690,22 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr"/>
-      <c r="M3" s="4" t="inlineStr"/>
+          <t>Sealed · pending grok route seal then authority model</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>pending_grok_route_seal_then_authority_model</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>grok_seal_pass_tasklet_fastlane</t>
+        </is>
+      </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>priority</t>
+          <t>review-safe-draft</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
@@ -707,29 +715,29 @@
       </c>
       <c r="P3" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Kakao Mobility (Kakao T)</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>kakao-mobility</t>
+          <t>hong-kong</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>super_app</t>
+          <t>destination_region</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>super_app</t>
+          <t>public_transit</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -739,12 +747,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Busan + the South-East coast; Jeju Island; Yeosu – Tongyeong (South Coast); Seoul — Han River + Incheon Bay</t>
+          <t>hong-kong, macau-china</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -781,19 +789,19 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>LINE (LY Corporation)</t>
+          <t>Kakao Mobility (Kakao T)</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>line</t>
+          <t>kakao-mobility</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -813,10 +821,14 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>network</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr"/>
+          <t>hub</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Busan + the South-East coast; Jeju Island; Yeosu – Tongyeong (South Coast); Seoul — Han River + Incheon Bay</t>
+        </is>
+      </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Open</t>
@@ -851,29 +863,29 @@
       </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Shun Tak / TurboJET</t>
+          <t>LINE (LY Corporation)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>shun-tak</t>
+          <t>line</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>ferry_operator</t>
+          <t>super_app</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>public_transit</t>
+          <t>super_app</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -883,14 +895,10 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>single</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>hong-kong, macau-china</t>
-        </is>
-      </c>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Open</t>
@@ -915,7 +923,7 @@
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>flagship</t>
+          <t>priority</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -925,34 +933,34 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>D-Marin</t>
+          <t>Shun Tak / TurboJET</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>d-marin</t>
+          <t>shun-tak</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>marina_network</t>
+          <t>ferry_operator</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>hospitality</t>
+          <t>public_transit</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>East Asia</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -962,7 +970,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>split-croatia, athens-saronic-greece, bodrum-turkey, dubai-uae</t>
+          <t>hong-kong, macau-china</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -999,29 +1007,29 @@
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>FREENOW</t>
+          <t>D-Marin</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>freenow</t>
+          <t>d-marin</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>marina_network</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>hospitality</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1031,12 +1039,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>France coastal; Greece coastal; Ireland coastal; Italy coastal; Spain coastal; United Kingdom coastal</t>
+          <t>split-croatia, athens-saronic-greece, bodrum-turkey, dubai-uae</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -1061,7 +1069,11 @@
       </c>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>flagship</t>
+        </is>
+      </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
           <t>partner-pitch</t>
@@ -1069,29 +1081,29 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Fjord Norway</t>
+          <t>FREENOW</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>norway-fjords</t>
+          <t>freenow</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>destination_region</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>public_transit</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -1101,12 +1113,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>hub</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>geiranger-norway, bergen-norway, stavanger-norway</t>
+          <t>France coastal; Greece coastal; Ireland coastal; Italy coastal; Spain coastal; United Kingdom coastal</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1131,11 +1143,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr"/>
       <c r="M9" s="4" t="inlineStr"/>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t>flagship</t>
-        </is>
-      </c>
+      <c r="N9" s="4" t="inlineStr"/>
       <c r="O9" s="4" t="inlineStr">
         <is>
           <t>partner-pitch</t>
@@ -1143,44 +1151,44 @@
       </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Cabify</t>
+          <t>Fjord Norway</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>cabify</t>
+          <t>norway-fjords</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>destination_region</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>public_transit</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Europe + LatAm</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Spain coastal; Colombia coastal</t>
+          <t>geiranger-norway, bergen-norway, stavanger-norway</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -1205,7 +1213,11 @@
       </c>
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>flagship</t>
+        </is>
+      </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
           <t>partner-pitch</t>
@@ -1213,44 +1225,44 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Thames Clippers / TfL</t>
+          <t>Cabify</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>thames-clippers</t>
+          <t>cabify</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>ferry_operator</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>public_transit</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Europe / Med</t>
+          <t>Europe + LatAm</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>hub</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>london-thames-uk</t>
+          <t>Spain coastal; Colombia coastal</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1275,11 +1287,7 @@
       </c>
       <c r="L11" s="4" t="inlineStr"/>
       <c r="M11" s="4" t="inlineStr"/>
-      <c r="N11" s="4" t="inlineStr">
-        <is>
-          <t>priority</t>
-        </is>
-      </c>
+      <c r="N11" s="4" t="inlineStr"/>
       <c r="O11" s="4" t="inlineStr">
         <is>
           <t>partner-pitch</t>
@@ -1287,44 +1295,44 @@
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Aman</t>
+          <t>Thames Clippers / TfL</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>aman</t>
+          <t>thames-clippers</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>hospitality_brand</t>
+          <t>ferry_operator</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>hospitality</t>
+          <t>public_transit</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Europe / Med</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Venice (Aman Venice); Philippines (Amanpulo); Indonesia (Amankila / Amanwana); Thailand — Amanpuri; Montenegro — Aman Sveti Stefan; Greece — Amanzoe</t>
+          <t>london-thames-uk</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -1351,7 +1359,7 @@
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>flagship</t>
+          <t>priority</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1361,24 +1369,24 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Discovery Land Company</t>
+          <t>Aman</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>discovery-land</t>
+          <t>aman</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>luxury_portfolio</t>
+          <t>hospitality_brand</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1398,7 +1406,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Baker's Bay — Bahamas; Costa Palmas — Los Cabos; Barbuda Ocean Club — Caribbean</t>
+          <t>Venice (Aman Venice); Philippines (Amanpulo); Indonesia (Amankila / Amanwana); Thailand — Amanpuri; Montenegro — Aman Sveti Stefan; Greece — Amanzoe</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1435,24 +1443,24 @@
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Four Seasons</t>
+          <t>Discovery Land Company</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>four-seasons</t>
+          <t>discovery-land</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>hospitality_brand</t>
+          <t>luxury_portfolio</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1472,7 +1480,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Maldives; French Polynesia (Bora Bora); Seychelles; Thailand — Four Seasons Koh Samui; Indonesia — Four Seasons Bali; Mauritius — Four Seasons Anahita</t>
+          <t>Baker's Bay — Bahamas; Costa Palmas — Los Cabos; Barbuda Ocean Club — Caribbean</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -1480,9 +1488,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1509,19 +1517,19 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Six Senses</t>
+          <t>Four Seasons</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>six-senses</t>
+          <t>four-seasons</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1546,7 +1554,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Maldives (Six Senses Laamu); Seychelles (Six Senses Zil Pasyon); Vietnam (Six Senses Con Dao); Thailand — Six Senses Yao Noi; Oman — Six Senses Zighy Bay; Fiji — Six Senses Fiji</t>
+          <t>Maldives; French Polynesia (Bora Bora); Seychelles; Thailand — Four Seasons Koh Samui; Indonesia — Four Seasons Bali; Mauritius — Four Seasons Anahita</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1554,9 +1562,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1583,25 +1591,29 @@
       </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>Six Senses</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>uber</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
+          <t>six-senses</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>hospitality_brand</t>
+        </is>
+      </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>hospitality</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1616,7 +1628,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>MENA / Gulf; Miami / Florida; SF Bay Area; Hawaii; Mediterranean; Sydney / NSW; Brazil / LatAm; Italy luxury; Côte d'Azur</t>
+          <t>Maldives (Six Senses Laamu); Seychelles (Six Senses Zil Pasyon); Vietnam (Six Senses Con Dao); Thailand — Six Senses Yao Noi; Oman — Six Senses Zighy Bay; Fiji — Six Senses Fiji</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -1624,9 +1636,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1641,7 +1653,11 @@
       </c>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>flagship</t>
+        </is>
+      </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
           <t>partner-pitch</t>
@@ -1649,34 +1665,30 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Soneva</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>soneva</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>hospitality_brand</t>
-        </is>
-      </c>
+          <t>uber</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>hospitality</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Global (Maldives + Thailand)</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1686,7 +1698,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Maldives; Soneva Kiri (Eastern Gulf of Thailand)</t>
+          <t>MENA / Gulf; Miami / Florida; SF Bay Area; Hawaii; Mediterranean; Sydney / NSW; Brazil / LatAm; Italy luxury; Côte d'Azur; Kolkata / Hooghly waterfront; Chennai / ECR / Cuddalore / Puducherry coast</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -1694,9 +1706,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1711,11 +1723,7 @@
       </c>
       <c r="L17" s="4" t="inlineStr"/>
       <c r="M17" s="4" t="inlineStr"/>
-      <c r="N17" s="4" t="inlineStr">
-        <is>
-          <t>flagship</t>
-        </is>
-      </c>
+      <c r="N17" s="4" t="inlineStr"/>
       <c r="O17" s="4" t="inlineStr">
         <is>
           <t>partner-pitch</t>
@@ -1723,34 +1731,34 @@
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>InDrive</t>
+          <t>Soneva</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>indrive</t>
+          <t>soneva</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>hospitality_brand</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>hospitality</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Global South (MENA · Africa · South Asia · LatAm)</t>
+          <t>Global (Maldives + Thailand)</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1760,7 +1768,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Egypt — Red Sea (Hurghada / El Gouna ↔ Sharm); Morocco — Atlantic (Agadir ↔ Essaouira); India (Mumbai &amp; Goa); Sub-Saharan Africa (Lagos · Cape Town · Zanzibar)</t>
+          <t>Maldives; Soneva Kiri (Eastern Gulf of Thailand)</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -1787,7 +1795,7 @@
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>priority</t>
+          <t>flagship</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -1797,19 +1805,19 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>DiDi</t>
+          <t>InDrive</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>didi</t>
+          <t>indrive</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1824,7 +1832,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>LatAm + Global South</t>
+          <t>Global South (MENA · Africa · South Asia · LatAm)</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1834,7 +1842,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Brazil; Mexico — Pacific (Los Cabos &amp; Puerto Vallarta); Mexico — Caribbean (Cancún &amp; Riviera Maya); Colombia (Cartagena &amp; the Rosario Islands); Panama (San Blas / Guna Yala); Costa Rica (Papagayo &amp; Nicoya); Dominican Republic (Samaná)</t>
+          <t>Egypt — Red Sea (Hurghada / El Gouna ↔ Sharm); Morocco — Atlantic (Agadir ↔ Essaouira); India (Mumbai &amp; Goa); Sub-Saharan Africa (Lagos · Cape Town · Zanzibar)</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -1871,44 +1879,44 @@
       </c>
       <c r="P19" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Abu Dhabi ITC</t>
+          <t>DiDi</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>abu-dhabi-itc</t>
+          <t>didi</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>transit_authority</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>public_transit</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>MENA</t>
+          <t>LatAm + Global South</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>hub</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>abu-dhabi-uae, dubai-uae</t>
+          <t>Brazil; Mexico — Pacific (Los Cabos &amp; Puerto Vallarta); Mexico — Caribbean (Cancún &amp; Riviera Maya); Colombia (Cartagena &amp; the Rosario Islands); Panama (San Blas / Guna Yala); Costa Rica (Papagayo &amp; Nicoya); Dominican Republic (Samaná)</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -1945,29 +1953,29 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Careem</t>
+          <t>Abu Dhabi ITC</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>careem</t>
+          <t>abu-dhabi-itc</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>super_app</t>
+          <t>transit_authority</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>super_app</t>
+          <t>public_transit</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1982,7 +1990,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>dubai-uae, abu-dhabi-uae, sharjah-uae, ras-al-khaimah-uae, fujairah-uae, manama-bahrain, doha-qatar, khasab-oman</t>
+          <t>abu-dhabi-uae, dubai-uae</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -1990,9 +1998,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2002,14 +2010,10 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>cascaded</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>cascaded</t>
-        </is>
-      </c>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr"/>
       <c r="M21" s="4" t="inlineStr"/>
       <c r="N21" s="4" t="inlineStr">
         <is>
@@ -2023,29 +2027,29 @@
       </c>
       <c r="P21" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Dubai RTA</t>
+          <t>Careem</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>dubai-rta</t>
+          <t>careem</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>transit_authority</t>
+          <t>super_app</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>public_transit</t>
+          <t>super_app</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -2060,7 +2064,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>dubai-uae, abu-dhabi-uae, fujairah-uae, ras-al-khaimah-uae, sharjah-uae</t>
+          <t>dubai-uae, abu-dhabi-uae, sharjah-uae, ras-al-khaimah-uae, fujairah-uae, manama-bahrain, doha-qatar, khasab-oman</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -2068,9 +2072,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2080,14 +2084,18 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr"/>
+          <t>cascaded</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>cascaded</t>
+        </is>
+      </c>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>flagship</t>
+          <t>priority</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
@@ -2097,29 +2105,29 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Noon</t>
+          <t>Dubai RTA</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>noon</t>
+          <t>dubai-rta</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>commerce_logistics_superapp</t>
+          <t>transit_authority</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>super_app</t>
+          <t>public_transit</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -2134,7 +2142,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>abu-dhabi-uae, dubai-uae, fujairah-uae, ras-al-khaimah-uae, sharjah-uae, doha-qatar, manama-bahrain, muscat-oman</t>
+          <t>dubai-uae, abu-dhabi-uae, fujairah-uae, ras-al-khaimah-uae, sharjah-uae</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2142,9 +2150,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2154,18 +2162,14 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>cascaded · Review tier</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>cascaded</t>
-        </is>
-      </c>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr"/>
       <c r="M23" s="4" t="inlineStr"/>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>flagship</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
@@ -2175,29 +2179,29 @@
       </c>
       <c r="P23" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Qatar Tourism</t>
+          <t>Noon</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>qatar</t>
+          <t>noon</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>transit_authority</t>
+          <t>commerce_logistics_superapp</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>public_transit</t>
+          <t>super_app</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -2212,7 +2216,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>doha-qatar, manama-bahrain</t>
+          <t>abu-dhabi-uae, dubai-uae, fujairah-uae, ras-al-khaimah-uae, sharjah-uae, doha-qatar, manama-bahrain, muscat-oman</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -2232,7 +2236,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>cascaded</t>
+          <t>cascaded · Review tier</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -2243,7 +2247,7 @@
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>priority</t>
+          <t>review</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -2253,29 +2257,29 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Red Sea Global</t>
+          <t>Qatar Tourism</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>red-sea-global</t>
+          <t>qatar</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>sovereign_developer</t>
+          <t>transit_authority</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>hospitality</t>
+          <t>public_transit</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -2290,7 +2294,7 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>red-sea-global-ksa, neom-sindalah-ksa, jeddah-ksa</t>
+          <t>doha-qatar, manama-bahrain</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -2310,14 +2314,18 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr"/>
+          <t>cascaded</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>cascaded</t>
+        </is>
+      </c>
       <c r="M25" s="4" t="inlineStr"/>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>flagship</t>
+          <t>priority</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
@@ -2327,19 +2335,19 @@
       </c>
       <c r="P25" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia (PIF)</t>
+          <t>Red Sea Global</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>saudi-pif</t>
+          <t>red-sea-global</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2349,7 +2357,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>sovereign</t>
+          <t>hospitality</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -2364,7 +2372,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>red-sea-global-ksa, neom-sindalah-ksa, jeddah-ksa, eastern-province-ksa</t>
+          <t>red-sea-global-ksa, neom-sindalah-ksa, jeddah-ksa</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -2391,7 +2399,7 @@
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>priority</t>
+          <t>flagship</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
@@ -2401,40 +2409,44 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Yango</t>
+          <t>Saudi Arabia (PIF)</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>yango</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr"/>
+          <t>saudi-pif</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>sovereign_developer</t>
+        </is>
+      </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>sovereign</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>MENA + Africa</t>
+          <t>MENA</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>UAE (Dubai + Abu Dhabi); West Africa (Lagos)</t>
+          <t>red-sea-global-ksa, neom-sindalah-ksa, jeddah-ksa, eastern-province-ksa</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -2459,7 +2471,11 @@
       </c>
       <c r="L27" s="4" t="inlineStr"/>
       <c r="M27" s="4" t="inlineStr"/>
-      <c r="N27" s="4" t="inlineStr"/>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
           <t>partner-pitch</t>
@@ -2467,44 +2483,40 @@
       </c>
       <c r="P27" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>BC Ferries</t>
+          <t>Yango</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>bc-ferries</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>ferry_operator</t>
-        </is>
-      </c>
+          <t>yango</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>public_transit</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>MENA + Africa</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>hub</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>vancouver-canada</t>
+          <t>UAE (Dubai + Abu Dhabi); West Africa (Lagos)</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -2512,9 +2524,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2529,11 +2541,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr">
-        <is>
-          <t>priority</t>
-        </is>
-      </c>
+      <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr">
         <is>
           <t>partner-pitch</t>
@@ -2541,24 +2549,24 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Hawaiʻi — Pulama Lānaʻi × DOT Harbors</t>
+          <t>BC Ferries</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>hawaii</t>
+          <t>bc-ferries</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>destination_region</t>
+          <t>ferry_operator</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -2578,7 +2586,7 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>maui-county-hawaii-usa, kona-hilo-hawaii-island-usa, oahu-honolulu-hawaii-usa, kauai-hawaii-usa</t>
+          <t>vancouver-canada</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -2615,29 +2623,29 @@
       </c>
       <c r="P29" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Lyft</t>
+          <t>Hawaiʻi — Pulama Lānaʻi × DOT Harbors</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>lyft</t>
+          <t>hawaii</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>destination_region</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>public_transit</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2647,12 +2655,12 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>New York; Miami &amp; South Florida; San Francisco Bay Area; Seattle &amp; Puget Sound; Boston &amp; New England; Athens &amp; the Cyclades</t>
+          <t>maui-county-hawaii-usa, kona-hilo-hawaii-island-usa, oahu-honolulu-hawaii-usa, kauai-hawaii-usa</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -2689,29 +2697,29 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>NYC Ferry</t>
+          <t>Lyft</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>nyc-ferry</t>
+          <t>lyft</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>ferry_operator</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>public_transit</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -2721,12 +2729,12 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>hub</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>new-york-harbor-usa</t>
+          <t>New York; Miami &amp; South Florida; San Francisco Bay Area; Seattle &amp; Puget Sound; Boston &amp; New England; Athens &amp; the Cyclades</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -2763,19 +2771,19 @@
       </c>
       <c r="P31" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Washington State Ferries</t>
+          <t>NYC Ferry</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>wsf</t>
+          <t>nyc-ferry</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2800,7 +2808,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>seattle-puget-sound-usa</t>
+          <t>new-york-harbor-usa</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -2837,19 +2845,19 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Fullers360</t>
+          <t>Washington State Ferries</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>fullers360</t>
+          <t>wsf</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2864,7 +2872,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Oceania</t>
+          <t>North America</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2874,7 +2882,7 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>auckland-new-zealand</t>
+          <t>seattle-puget-sound-usa</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
@@ -2911,24 +2919,24 @@
       </c>
       <c r="P33" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Transport for NSW</t>
+          <t>Fullers360</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>transport-nsw</t>
+          <t>fullers360</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>transit_authority</t>
+          <t>ferry_operator</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2948,7 +2956,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>sydney-australia</t>
+          <t>auckland-new-zealand</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -2985,44 +2993,44 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Gojek (GoTo)</t>
+          <t>Transport for NSW</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>gojek</t>
+          <t>transport-nsw</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>super_app</t>
+          <t>transit_authority</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>super_app</t>
+          <t>public_transit</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>Oceania</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Jakarta; Bali, Nusa &amp; the Gili Islands; Komodo &amp; Flores; Riau Islands ↔ Singapore; Singapore; Eastern Indonesia Frontier</t>
+          <t>sydney-australia</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
@@ -3059,22 +3067,26 @@
       </c>
       <c r="P35" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Grab</t>
+          <t>Gojek (GoTo)</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>grab</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr"/>
+          <t>gojek</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>super_app</t>
+        </is>
+      </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
           <t>super_app</t>
@@ -3092,7 +3104,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Singapore; Cross-border crossings; Bali + the luxury island chain; Phuket + the Andaman; Philippines; Vietnam</t>
+          <t>Jakarta; Bali, Nusa &amp; the Gili Islands; Komodo &amp; Flores; Riau Islands ↔ Singapore; Singapore; Eastern Indonesia Frontier</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -3100,9 +3112,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I36" s="3" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3117,7 +3129,11 @@
       </c>
       <c r="L36" s="2" t="inlineStr"/>
       <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
           <t>partner-pitch</t>
@@ -3125,29 +3141,25 @@
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Singapore MPA</t>
+          <t>Grab</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>singapore-mpa</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>transit_authority</t>
-        </is>
-      </c>
+          <t>grab</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr"/>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>public_transit</t>
+          <t>super_app</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -3157,12 +3169,12 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>hub</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>singapore, riau-islands-indonesia, desaru-coast-malaysia</t>
+          <t>Singapore; Cross-border crossings; Bali + the luxury island chain; Phuket + the Andaman; Philippines; Vietnam</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
@@ -3170,9 +3182,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3187,11 +3199,7 @@
       </c>
       <c r="L37" s="4" t="inlineStr"/>
       <c r="M37" s="4" t="inlineStr"/>
-      <c r="N37" s="4" t="inlineStr">
-        <is>
-          <t>priority</t>
-        </is>
-      </c>
+      <c r="N37" s="4" t="inlineStr"/>
       <c r="O37" s="4" t="inlineStr">
         <is>
           <t>partner-pitch</t>
@@ -3199,44 +3207,44 @@
       </c>
       <c r="P37" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Adani Ports &amp; SEZ</t>
+          <t>Singapore MPA</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>adani-ports</t>
+          <t>singapore-mpa</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>india_water_mobility_operator</t>
+          <t>transit_authority</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>corporate</t>
+          <t>public_transit</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>South Asia</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Mumbai &amp; the Konkan coast; Goa — rivers, coast &amp; islands; Kerala — Kochi, Vizhinjam &amp; the backwaters; Andaman &amp; Nicobar island network; Kolkata / Hooghly waterfront; Chennai / ECR / Cuddalore / Puducherry coast</t>
+          <t>singapore, riau-islands-indonesia, desaru-coast-malaysia</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
@@ -3256,22 +3264,14 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Sealed · not run no source demand fare yet · Review tier</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>not_run_no_source_demand_fare_yet</t>
-        </is>
-      </c>
-      <c r="M38" s="2" t="inlineStr">
-        <is>
-          <t>grok_seal_pass_pr61</t>
-        </is>
-      </c>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>priority</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
@@ -3281,29 +3281,29 @@
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Constance Hotels &amp; Resorts</t>
+          <t>Adani Ports &amp; SEZ</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>constance</t>
+          <t>adani-ports</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>hospitality_brand</t>
+          <t>india_water_mobility_operator</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>hospitality</t>
+          <t>corporate</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -3313,12 +3313,12 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>hub</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>male-maldives</t>
+          <t>Mumbai &amp; the Konkan coast; Goa — rivers, coast &amp; islands; Kerala — Kochi, Vizhinjam &amp; the backwaters; Andaman &amp; Nicobar island network; Kolkata / Hooghly waterfront; Chennai / ECR / Cuddalore / Puducherry coast</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
@@ -3326,9 +3326,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I39" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3338,14 +3338,22 @@
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="L39" s="4" t="inlineStr"/>
-      <c r="M39" s="4" t="inlineStr"/>
+          <t>Sealed · not run no source demand fare yet · Review tier</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>not_run_no_source_demand_fare_yet</t>
+        </is>
+      </c>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t>grok_seal_pass_pr61</t>
+        </is>
+      </c>
       <c r="N39" s="4" t="inlineStr">
         <is>
-          <t>watch</t>
+          <t>review</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
@@ -3355,19 +3363,19 @@
       </c>
       <c r="P39" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Crown &amp; Champa Resorts</t>
+          <t>Constance Hotels &amp; Resorts</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>crown-champa</t>
+          <t>constance</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -3400,9 +3408,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -3429,29 +3437,29 @@
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>JIH Global</t>
+          <t>Crown &amp; Champa Resorts</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>jih-global</t>
+          <t>crown-champa</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>investment_jv</t>
+          <t>hospitality_brand</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>sovereign</t>
+          <t>hospitality</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -3474,9 +3482,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I41" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3486,18 +3494,14 @@
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>cascaded</t>
-        </is>
-      </c>
-      <c r="L41" s="4" t="inlineStr">
-        <is>
-          <t>cascaded</t>
-        </is>
-      </c>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr"/>
       <c r="M41" s="4" t="inlineStr"/>
       <c r="N41" s="4" t="inlineStr">
         <is>
-          <t>flagship</t>
+          <t>watch</t>
         </is>
       </c>
       <c r="O41" s="4" t="inlineStr">
@@ -3507,29 +3511,29 @@
       </c>
       <c r="P41" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Maldives</t>
+          <t>JIH Global</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>maldives</t>
+          <t>jih-global</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>destination_region</t>
+          <t>investment_jv</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>hospitality</t>
+          <t>sovereign</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -3552,9 +3556,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -3564,10 +3568,14 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr"/>
+          <t>cascaded</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>cascaded</t>
+        </is>
+      </c>
       <c r="M42" s="2" t="inlineStr"/>
       <c r="N42" s="2" t="inlineStr">
         <is>
@@ -3581,29 +3589,29 @@
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Maldives — National Ferry Network</t>
+          <t>Maldives</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>maldives-government</t>
+          <t>maldives</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>transit_authority</t>
+          <t>destination_region</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>public_transit</t>
+          <t>hospitality</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -3645,7 +3653,7 @@
       <c r="M43" s="4" t="inlineStr"/>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>priority</t>
+          <t>flagship</t>
         </is>
       </c>
       <c r="O43" s="4" t="inlineStr">
@@ -3655,29 +3663,29 @@
       </c>
       <c r="P43" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Ola</t>
+          <t>Maldives — National Ferry Network</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>ola</t>
+          <t>maldives-government</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>transit_authority</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>public_transit</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -3687,12 +3695,12 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Mumbai &amp; the Konkan coast; Goa - rivers, coast &amp; islands; Kerala - Kochi &amp; the backwaters; Andaman &amp; Nicobar Islands</t>
+          <t>male-maldives</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
@@ -3700,9 +3708,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I44" s="3" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -3712,14 +3720,10 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>cascaded</t>
-        </is>
-      </c>
-      <c r="L44" s="2" t="inlineStr">
-        <is>
-          <t>cascaded</t>
-        </is>
-      </c>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr"/>
       <c r="M44" s="2" t="inlineStr"/>
       <c r="N44" s="2" t="inlineStr">
         <is>
@@ -3733,19 +3737,19 @@
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Rapido</t>
+          <t>Ola</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>rapido</t>
+          <t>ola</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -3770,7 +3774,7 @@
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>Mumbai &amp; the Konkan coast; Goa - rivers, coast &amp; islands; Kerala - Kochi &amp; the backwaters; Andaman &amp; Nicobar Islands</t>
+          <t>Mumbai &amp; the Konkan coast; Goa - rivers, coast &amp; islands; Kerala - Kochi &amp; the backwaters; Andaman &amp; Nicobar Islands; Kolkata / Hooghly waterfront; Chennai / ECR / Cuddalore / Puducherry coast</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
@@ -3790,15 +3794,19 @@
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
+          <t>Sealed · cascaded</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
           <t>cascaded</t>
         </is>
       </c>
-      <c r="L45" s="4" t="inlineStr">
-        <is>
-          <t>cascaded</t>
-        </is>
-      </c>
-      <c r="M45" s="4" t="inlineStr"/>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>grok_seal_pass_tasklet_fastlane</t>
+        </is>
+      </c>
       <c r="N45" s="4" t="inlineStr">
         <is>
           <t>priority</t>
@@ -3811,29 +3819,29 @@
       </c>
       <c r="P45" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Reliance Industries</t>
+          <t>Rapido</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>reliance-industries</t>
+          <t>rapido</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>india_water_mobility_operator</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>corporate</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -3848,7 +3856,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Mumbai &amp; the Konkan coast; Goa — rivers, coast &amp; islands; Kerala — Kochi, Vizhinjam &amp; the backwaters; Andaman &amp; Nicobar island network; Kolkata / Hooghly waterfront; Chennai / ECR / Cuddalore / Puducherry coast</t>
+          <t>Mumbai &amp; the Konkan coast; Goa - rivers, coast &amp; islands; Kerala - Kochi &amp; the backwaters; Andaman &amp; Nicobar Islands; Kolkata / Hooghly waterfront; Chennai / ECR / Cuddalore / Puducherry coast</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
@@ -3856,9 +3864,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -3868,22 +3876,22 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Sealed · not run no source demand fare yet · Review tier</t>
+          <t>Sealed · cascaded</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>not_run_no_source_demand_fare_yet</t>
+          <t>cascaded</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>grok_seal_pass_pr61</t>
+          <t>grok_seal_pass_tasklet_fastlane</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>priority</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
@@ -3893,29 +3901,29 @@
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Sun Siyam Resorts</t>
+          <t>Reliance Industries</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>sun-siyam</t>
+          <t>reliance-industries</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>hospitality_brand</t>
+          <t>india_water_mobility_operator</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>hospitality</t>
+          <t>corporate</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -3925,12 +3933,12 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>hub</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>male-maldives</t>
+          <t>Mumbai &amp; the Konkan coast; Goa — rivers, coast &amp; islands; Kerala — Kochi, Vizhinjam &amp; the backwaters; Andaman &amp; Nicobar island network; Kolkata / Hooghly waterfront; Chennai / ECR / Cuddalore / Puducherry coast</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
@@ -3950,14 +3958,22 @@
       </c>
       <c r="K47" s="4" t="inlineStr">
         <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="L47" s="4" t="inlineStr"/>
-      <c r="M47" s="4" t="inlineStr"/>
+          <t>Sealed · not run no source demand fare yet · Review tier</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>not_run_no_source_demand_fare_yet</t>
+        </is>
+      </c>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>grok_seal_pass_pr61</t>
+        </is>
+      </c>
       <c r="N47" s="4" t="inlineStr">
         <is>
-          <t>watch</t>
+          <t>review</t>
         </is>
       </c>
       <c r="O47" s="4" t="inlineStr">
@@ -3967,29 +3983,29 @@
       </c>
       <c r="P47" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Uber India (draft)</t>
+          <t>Sun Siyam Resorts</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>uber-india-derivative</t>
+          <t>sun-siyam</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>hospitality_brand</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>hospitality</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -3999,12 +4015,12 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Mumbai &amp; the Konkan coast; Goa - rivers, coast &amp; islands; Kerala - Kochi &amp; the backwaters; Andaman &amp; Nicobar Islands</t>
+          <t>male-maldives</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
@@ -4024,46 +4040,46 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Economics pending</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>economics_pending</t>
-        </is>
-      </c>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr"/>
-      <c r="N48" s="2" t="inlineStr"/>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>partner-pitch</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Universal Resorts</t>
+          <t>Uber India (draft)</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>universal-enterprises</t>
+          <t>uber-india-derivative</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>luxury_portfolio</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>hospitality</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
@@ -4073,12 +4089,12 @@
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>hub</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>male-maldives</t>
+          <t>Mumbai &amp; the Konkan coast; Goa - rivers, coast &amp; islands; Kerala - Kochi &amp; the backwaters; Andaman &amp; Nicobar Islands</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
@@ -4098,36 +4114,36 @@
       </c>
       <c r="K49" s="4" t="inlineStr">
         <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="L49" s="4" t="inlineStr"/>
+          <t>Economics pending</t>
+        </is>
+      </c>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>economics_pending</t>
+        </is>
+      </c>
       <c r="M49" s="4" t="inlineStr"/>
-      <c r="N49" s="4" t="inlineStr">
-        <is>
-          <t>watch</t>
-        </is>
-      </c>
+      <c r="N49" s="4" t="inlineStr"/>
       <c r="O49" s="4" t="inlineStr">
         <is>
-          <t>partner-pitch</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="P49" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Villa Hotels &amp; Resorts</t>
+          <t>Universal Resorts</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>villa-hotels</t>
+          <t>universal-enterprises</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -4189,40 +4205,44 @@
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Bolt</t>
+          <t>Villa Hotels &amp; Resorts</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>bolt</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="inlineStr"/>
+          <t>villa-hotels</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>luxury_portfolio</t>
+        </is>
+      </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>ridehail</t>
+          <t>hospitality</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>europe-med</t>
+          <t>South Asia</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>hub</t>
+          <t>single</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>Greece — Athens, the Saronic &amp; the Cyclades; Croatia — the Dalmatian coast; Italy — Amalfi, Capri &amp; the Venice lagoon; France — the Côte d'Azur; UAE — Dubai &amp; Abu Dhabi; Saudi Arabia — Jeddah &amp; the Red Sea</t>
+          <t>male-maldives</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
@@ -4230,9 +4250,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I51" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr">
@@ -4247,7 +4267,11 @@
       </c>
       <c r="L51" s="4" t="inlineStr"/>
       <c r="M51" s="4" t="inlineStr"/>
-      <c r="N51" s="4" t="inlineStr"/>
+      <c r="N51" s="4" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
       <c r="O51" s="4" t="inlineStr">
         <is>
           <t>partner-pitch</t>
@@ -4255,34 +4279,34 @@
       </c>
       <c r="P51" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Côte d'Azur</t>
+          <t>RAKTA</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>cote-dazur</t>
+          <t>rakta</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>destination_region</t>
+          <t>Authority / public transport</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>hospitality</t>
+          <t>public_transit</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>europe-med</t>
+          <t>UAE / Northern Gulf</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -4292,7 +4316,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>cote-dazur-france, monaco-monaco</t>
+          <t>ras-al-khaimah-uae, dubai-uae, sharjah-uae, fujairah-uae, abu-dhabi-uae, muscat-oman, doha-qatar, manama-bahrain</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
@@ -4312,14 +4336,22 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="L52" s="2" t="inlineStr"/>
-      <c r="M52" s="2" t="inlineStr"/>
+          <t>Sealed · pending grok route seal then authority model</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>pending_grok_route_seal_then_authority_model</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>grok_seal_pass_tasklet_fastlane</t>
+        </is>
+      </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>priority</t>
+          <t>review-safe-draft</t>
         </is>
       </c>
       <c r="O52" s="2" t="inlineStr">
@@ -4329,44 +4361,40 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 04:22 UTC</t>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>French Polynesia</t>
+          <t>Bolt</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>french-polynesia</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>destination_region</t>
-        </is>
-      </c>
+          <t>bolt</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr"/>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>hospitality</t>
+          <t>ridehail</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>pacific</t>
+          <t>europe-med</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>hub</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>tahiti-moorea-french-polynesia, moorea-french-polynesia, bora-bora-french-polynesia, raiatea-tahaa-french-polynesia, huahine-french-polynesia, maupiti-french-polynesia, rangiroa-tuamotus-french-polynesia, marquesas-french-polynesia</t>
+          <t>Greece — Athens, the Saronic &amp; the Cyclades; Croatia — the Dalmatian coast; Italy — Amalfi, Capri &amp; the Venice lagoon; France — the Côte d'Azur; UAE — Dubai &amp; Abu Dhabi; Saudi Arabia — Jeddah &amp; the Red Sea</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
@@ -4374,9 +4402,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I53" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr">
@@ -4391,19 +4419,163 @@
       </c>
       <c r="L53" s="4" t="inlineStr"/>
       <c r="M53" s="4" t="inlineStr"/>
-      <c r="N53" s="4" t="inlineStr">
+      <c r="N53" s="4" t="inlineStr"/>
+      <c r="O53" s="4" t="inlineStr">
+        <is>
+          <t>partner-pitch</t>
+        </is>
+      </c>
+      <c r="P53" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-21 05:02 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Côte d'Azur</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>cote-dazur</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>destination_region</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>hospitality</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>europe-med</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>cote-dazur-france, monaco-monaco</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr"/>
+      <c r="N54" s="2" t="inlineStr">
         <is>
           <t>priority</t>
         </is>
       </c>
-      <c r="O53" s="4" t="inlineStr">
-        <is>
-          <t>partner-pitch</t>
-        </is>
-      </c>
-      <c r="P53" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-21 04:22 UTC</t>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>partner-pitch</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 05:02 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>French Polynesia</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>french-polynesia</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>destination_region</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>hospitality</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>pacific</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>tahiti-moorea-french-polynesia, moorea-french-polynesia, bora-bora-french-polynesia, raiatea-tahaa-french-polynesia, huahine-french-polynesia, maupiti-french-polynesia, rangiroa-tuamotus-french-polynesia, marquesas-french-polynesia</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr"/>
+      <c r="M55" s="4" t="inlineStr"/>
+      <c r="N55" s="4" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="O55" s="4" t="inlineStr">
+        <is>
+          <t>partner-pitch</t>
+        </is>
+      </c>
+      <c r="P55" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-21 05:02 UTC</t>
         </is>
       </c>
     </row>
@@ -4422,28 +4594,28 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId38"/>
@@ -4452,29 +4624,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(inheritance): regional spine system + Uber India consumer sync
- Apply regional inheritance manifest, inherit_regional_spine.py, spine parity gate
- Wire 8-step partner page lane (inherit bind → parity → relink → QA)
- Extend india_mobility brief_only markets; add gulf_authority pack (RAKTA/Bahrain MOTC)
- Sync Kolkata/Chennai into uber-india-derivative; promote from draft to live page
- QA geometry metric split; relink double-count fix retained
</commit_message>
<xml_diff>
--- a/finance/_partner-tracker.xlsx
+++ b/finance/_partner-tracker.xlsx
@@ -633,7 +633,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="P3" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
       </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1532,11 +1532,7 @@
           <t>four-seasons</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>hospitality_brand</t>
-        </is>
-      </c>
+      <c r="C15" s="4" t="inlineStr"/>
       <c r="D15" s="4" t="inlineStr">
         <is>
           <t>hospitality</t>
@@ -1554,7 +1550,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Maldives; French Polynesia (Bora Bora); Seychelles; Thailand — Four Seasons Koh Samui; Indonesia — Four Seasons Bali; Mauritius — Four Seasons Anahita</t>
+          <t>Maldives; French Polynesia (Bora Bora); Seychelles</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1579,11 +1575,7 @@
       </c>
       <c r="L15" s="4" t="inlineStr"/>
       <c r="M15" s="4" t="inlineStr"/>
-      <c r="N15" s="4" t="inlineStr">
-        <is>
-          <t>flagship</t>
-        </is>
-      </c>
+      <c r="N15" s="4" t="inlineStr"/>
       <c r="O15" s="4" t="inlineStr">
         <is>
           <t>partner-pitch</t>
@@ -1591,7 +1583,7 @@
       </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1657,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1723,7 @@
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1797,7 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1871,7 @@
       </c>
       <c r="P19" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1945,7 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2019,7 @@
       </c>
       <c r="P21" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2056,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>dubai-uae, abu-dhabi-uae, sharjah-uae, ras-al-khaimah-uae, fujairah-uae, manama-bahrain, doha-qatar, khasab-oman</t>
+          <t>abu-dhabi-uae, dubai-uae, fujairah-uae, ras-al-khaimah-uae, sharjah-uae, doha-qatar, manama-bahrain, muscat-oman</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -2105,7 +2097,7 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2171,7 @@
       </c>
       <c r="P23" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2236,12 +2228,12 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>cascaded · Review tier</t>
+          <t>Economics pending · Review tier</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>cascaded</t>
+          <t>economics_pending</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr"/>
@@ -2257,7 +2249,7 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2327,7 @@
       </c>
       <c r="P25" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2401,7 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2424,11 +2416,7 @@
           <t>saudi-pif</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>sovereign_developer</t>
-        </is>
-      </c>
+      <c r="C27" s="4" t="inlineStr"/>
       <c r="D27" s="4" t="inlineStr">
         <is>
           <t>sovereign</t>
@@ -2471,11 +2459,7 @@
       </c>
       <c r="L27" s="4" t="inlineStr"/>
       <c r="M27" s="4" t="inlineStr"/>
-      <c r="N27" s="4" t="inlineStr">
-        <is>
-          <t>priority</t>
-        </is>
-      </c>
+      <c r="N27" s="4" t="inlineStr"/>
       <c r="O27" s="4" t="inlineStr">
         <is>
           <t>partner-pitch</t>
@@ -2483,7 +2467,7 @@
       </c>
       <c r="P27" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2549,7 +2533,7 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2623,7 +2607,7 @@
       </c>
       <c r="P29" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2681,7 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2755,7 @@
       </c>
       <c r="P31" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2829,7 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2919,7 +2903,7 @@
       </c>
       <c r="P33" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -2993,7 +2977,7 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3051,7 @@
       </c>
       <c r="P35" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3125,7 @@
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3191,7 @@
       </c>
       <c r="P37" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3265,7 @@
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3363,7 +3347,7 @@
       </c>
       <c r="P39" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3437,7 +3421,7 @@
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3495,7 @@
       </c>
       <c r="P41" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3568,14 +3552,10 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>cascaded</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>cascaded</t>
-        </is>
-      </c>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr"/>
       <c r="M42" s="2" t="inlineStr"/>
       <c r="N42" s="2" t="inlineStr">
         <is>
@@ -3589,7 +3569,7 @@
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3663,7 +3643,7 @@
       </c>
       <c r="P43" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3737,7 +3717,7 @@
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3819,7 +3799,7 @@
       </c>
       <c r="P45" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3881,7 @@
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3983,7 +3963,7 @@
       </c>
       <c r="P47" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -4057,14 +4037,14 @@
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Uber India (draft)</t>
+          <t>Uber India</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -4094,7 +4074,7 @@
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>Mumbai &amp; the Konkan coast; Goa - rivers, coast &amp; islands; Kerala - Kochi &amp; the backwaters; Andaman &amp; Nicobar Islands</t>
+          <t>Mumbai &amp; the Konkan coast; Goa - rivers, coast &amp; islands; Kerala - Kochi &amp; the backwaters; Andaman &amp; Nicobar Islands; Kolkata / Hooghly waterfront; Chennai / ECR / Cuddalore / Puducherry coast</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
@@ -4114,7 +4094,7 @@
       </c>
       <c r="K49" s="4" t="inlineStr">
         <is>
-          <t>Economics pending</t>
+          <t>Sealed · Economics pending</t>
         </is>
       </c>
       <c r="L49" s="4" t="inlineStr">
@@ -4122,16 +4102,20 @@
           <t>economics_pending</t>
         </is>
       </c>
-      <c r="M49" s="4" t="inlineStr"/>
+      <c r="M49" s="4" t="inlineStr">
+        <is>
+          <t>grok_seal_pass_tasklet_fastlane</t>
+        </is>
+      </c>
       <c r="N49" s="4" t="inlineStr"/>
       <c r="O49" s="4" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>partner-pitch</t>
         </is>
       </c>
       <c r="P49" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -4205,7 +4189,7 @@
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -4279,7 +4263,7 @@
       </c>
       <c r="P51" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -4361,7 +4345,7 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4411,7 @@
       </c>
       <c r="P53" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4485,7 @@
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>
@@ -4575,7 +4559,7 @@
       </c>
       <c r="P55" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:02 UTC</t>
+          <t>2026-06-21 05:08 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(inheritance): re-bind India partners after regional spine lane
Re-run inherit → relink → QA for rapido, ola, uber-india-derivative,
adani-ports, reliance-industries, and uber. Kolkata/Chennai remain
brief-only until Atlas city IDs are minted.
</commit_message>
<xml_diff>
--- a/finance/_partner-tracker.xlsx
+++ b/finance/_partner-tracker.xlsx
@@ -633,7 +633,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="P3" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
       </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="P19" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="P21" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="P23" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="P25" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="P27" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="P29" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="P31" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="P33" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="P35" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="P37" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="P39" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
       </c>
       <c r="P41" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3569,7 +3569,7 @@
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
       </c>
       <c r="P43" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="P45" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3963,7 @@
       </c>
       <c r="P47" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4115,7 +4115,7 @@
       </c>
       <c r="P49" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4189,7 +4189,7 @@
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4263,7 @@
       </c>
       <c r="P51" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4345,7 +4345,7 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="P53" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4485,7 +4485,7 @@
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="P55" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:08 UTC</t>
+          <t>2026-06-21 05:13 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(india): mint Kolkata/Chennai geometry, seal all India partners, Uber India live
- Mint kolkata-india + chennai-india cities, 8 ferry BPs, 5 routes
- Promote brief markets to sealed display on rapido/ola/uber-india/adani/reliance/uber
- Update regional inheritance manifest (6 display markets, 6 map-scope cities)
- Clean Uber India draft copy; add /uber-india → /uber-india-derivative redirect
- Kolkata/Chennai sub-pages now build on all India partners (12 new market pages)
</commit_message>
<xml_diff>
--- a/finance/_partner-tracker.xlsx
+++ b/finance/_partner-tracker.xlsx
@@ -633,7 +633,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="P3" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
       </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="P19" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="P21" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="P23" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="P25" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="P27" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="P29" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="P31" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="P33" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="P35" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="P37" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="P39" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
       </c>
       <c r="P41" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -3569,7 +3569,7 @@
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
       </c>
       <c r="P43" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="P45" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3963,7 @@
       </c>
       <c r="P47" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -4115,7 +4115,7 @@
       </c>
       <c r="P49" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -4189,7 +4189,7 @@
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4263,7 @@
       </c>
       <c r="P51" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -4345,7 +4345,7 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="P53" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -4485,7 +4485,7 @@
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="P55" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:13 UTC</t>
+          <t>2026-06-21 05:20 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(authority+india): expand RAK/Bahrain spine seal, India extensions + econ stubs
- Audit clarifies 6/10 fastlane vs 60/101 full spine coverage
- Expand RAK phase-1 (+8) and Bahrain phase-1 (+10) featured routes from spine
- Mint India extension routes (heritage, Chandannagar, Puducherry, Buckingham roadmap)
- Wire 9 india_kcc economics pending stubs; bind extension journeys on all India partners
</commit_message>
<xml_diff>
--- a/finance/_partner-tracker.xlsx
+++ b/finance/_partner-tracker.xlsx
@@ -633,7 +633,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="P3" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
       </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="P19" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="P21" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="P23" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="P25" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="P27" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="P29" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="P31" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="P33" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="P35" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="P37" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="P39" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
       </c>
       <c r="P41" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -3569,7 +3569,7 @@
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
       </c>
       <c r="P43" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="P45" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3963,7 @@
       </c>
       <c r="P47" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -4115,7 +4115,7 @@
       </c>
       <c r="P49" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -4189,7 +4189,7 @@
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4263,7 @@
       </c>
       <c r="P51" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -4345,7 +4345,7 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="P53" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -4485,7 +4485,7 @@
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="P55" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:20 UTC</t>
+          <t>2026-06-21 05:27 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(auto-lanes): post-merge orchestrator, full authority finance + spine expand
Wire run_post_merge_lane.sh as canonical post-Tasklet entry; fastlane chains to it.
Fix RAK Dubai contamination via label-first city inference (52 sealed featured cards).
Expand Bahrain to 94 sealed cards; finance cascade with Sheets, growth blocks, agg-global sidecar.
Register rakta, bahrain-motc, uber-india-derivative in PARTNER-SHEET-IDS; document auto-lane DAG.
</commit_message>
<xml_diff>
--- a/finance/_partner-tracker.xlsx
+++ b/finance/_partner-tracker.xlsx
@@ -633,7 +633,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -678,9 +678,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="P3" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
       </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="P19" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="P21" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="P23" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2228,12 +2228,12 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Economics pending · Review tier</t>
+          <t>cascaded · Review tier</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>economics_pending</t>
+          <t>cascaded</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr"/>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="P25" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="P27" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="P29" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="P31" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="P33" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="P35" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="P37" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="P39" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
       </c>
       <c r="P41" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3552,10 +3552,14 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr"/>
+          <t>cascaded</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>cascaded</t>
+        </is>
+      </c>
       <c r="M42" s="2" t="inlineStr"/>
       <c r="N42" s="2" t="inlineStr">
         <is>
@@ -3569,7 +3573,7 @@
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3647,7 @@
       </c>
       <c r="P43" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3721,7 @@
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3803,7 @@
       </c>
       <c r="P45" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3885,7 @@
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3967,7 @@
       </c>
       <c r="P47" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4041,7 @@
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -4082,9 +4086,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I49" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
@@ -4115,7 +4119,7 @@
       </c>
       <c r="P49" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -4189,7 +4193,7 @@
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4267,7 @@
       </c>
       <c r="P51" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -4308,9 +4312,9 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -4345,7 +4349,7 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4415,7 @@
       </c>
       <c r="P53" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -4485,7 +4489,7 @@
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4563,7 @@
       </c>
       <c r="P55" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21 05:27 UTC</t>
+          <t>2026-06-21 05:40 UTC</t>
         </is>
       </c>
     </row>
@@ -4567,72 +4571,75 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId71"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>